<commit_message>
Separated north and south italy
</commit_message>
<xml_diff>
--- a/Manuscript/Contributors.xlsx
+++ b/Manuscript/Contributors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10709"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/x0504807/Documents/Research/SpurginBosse_Hapmap/Manuscript/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lewisspurgin/Documents/Research/SpurginBosse_Hapmap/Manuscript/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5497C5E5-C6E4-8D42-BDFF-0D05354F920F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{B50FE7FE-2B73-B244-A7FC-22B97CE376E5}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1240" yWindow="460" windowWidth="32580" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="540" yWindow="2080" windowWidth="25600" windowHeight="11960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="129">
   <si>
     <t>Adriaensen Frank &lt;frank.adriaensen@uantwerpen.be&gt;,</t>
   </si>
@@ -243,15 +243,6 @@
     <t>Comment</t>
   </si>
   <si>
-    <t>Email returned</t>
-  </si>
-  <si>
-    <t>Away until 15/01/2019</t>
-  </si>
-  <si>
-    <t>Away until 22/01/2019</t>
-  </si>
-  <si>
     <t>Responded</t>
   </si>
   <si>
@@ -415,6 +406,12 @@
   </si>
   <si>
     <t>ebelda@dca.upv.es</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
 </sst>
 </file>
@@ -764,16 +761,16 @@
         <v>71</v>
       </c>
       <c r="D1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -783,11 +780,14 @@
       <c r="B2" t="s">
         <v>0</v>
       </c>
+      <c r="C2" t="s">
+        <v>127</v>
+      </c>
       <c r="D2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -797,11 +797,14 @@
       <c r="B3" t="s">
         <v>30</v>
       </c>
+      <c r="C3" t="s">
+        <v>128</v>
+      </c>
       <c r="D3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -811,25 +814,31 @@
       <c r="B4" t="s">
         <v>31</v>
       </c>
+      <c r="C4" t="s">
+        <v>128</v>
+      </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" t="s">
+        <v>126</v>
+      </c>
+      <c r="C5" t="s">
         <v>128</v>
       </c>
-      <c r="B5" t="s">
-        <v>129</v>
-      </c>
       <c r="D5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -839,11 +848,14 @@
       <c r="B6" t="s">
         <v>1</v>
       </c>
+      <c r="C6" t="s">
+        <v>128</v>
+      </c>
       <c r="D6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -853,11 +865,14 @@
       <c r="B7" t="s">
         <v>2</v>
       </c>
+      <c r="C7" t="s">
+        <v>127</v>
+      </c>
       <c r="D7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -867,11 +882,8 @@
       <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C8" t="s">
-        <v>74</v>
-      </c>
       <c r="E8" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -882,10 +894,10 @@
         <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -896,10 +908,10 @@
         <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -910,13 +922,13 @@
         <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F11" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -927,10 +939,10 @@
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E12" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -941,27 +953,27 @@
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E13" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>72</v>
+        <v>128</v>
       </c>
       <c r="D14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E14" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -971,11 +983,14 @@
       <c r="B15" t="s">
         <v>10</v>
       </c>
+      <c r="C15" t="s">
+        <v>127</v>
+      </c>
       <c r="D15" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -986,10 +1001,10 @@
         <v>11</v>
       </c>
       <c r="D16" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E16" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -999,11 +1014,14 @@
       <c r="B17" t="s">
         <v>13</v>
       </c>
+      <c r="C17" t="s">
+        <v>127</v>
+      </c>
       <c r="D17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E17" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1014,10 +1032,10 @@
         <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E18" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1027,34 +1045,31 @@
       <c r="B19" t="s">
         <v>14</v>
       </c>
-      <c r="C19" t="s">
-        <v>73</v>
-      </c>
       <c r="D19" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E19" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="F19" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G19" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B20" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D20" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E20" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1065,10 +1080,10 @@
         <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E21" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1079,10 +1094,10 @@
         <v>16</v>
       </c>
       <c r="D22" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E22" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1093,10 +1108,10 @@
         <v>17</v>
       </c>
       <c r="D23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E23" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1107,24 +1122,24 @@
         <v>18</v>
       </c>
       <c r="D24" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E24" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B25" t="s">
         <v>19</v>
       </c>
       <c r="D25" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E25" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1134,11 +1149,14 @@
       <c r="B26" t="s">
         <v>20</v>
       </c>
+      <c r="C26" t="s">
+        <v>127</v>
+      </c>
       <c r="D26" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E26" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1149,38 +1167,38 @@
         <v>21</v>
       </c>
       <c r="D27" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E27" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B28" t="s">
         <v>33</v>
       </c>
       <c r="D28" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B29" t="s">
         <v>22</v>
       </c>
       <c r="D29" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E29" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -1191,10 +1209,10 @@
         <v>23</v>
       </c>
       <c r="D30" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E30" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1205,13 +1223,13 @@
         <v>34</v>
       </c>
       <c r="D31" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E31" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F31" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1222,10 +1240,10 @@
         <v>35</v>
       </c>
       <c r="D32" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E32" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -1236,10 +1254,10 @@
         <v>24</v>
       </c>
       <c r="D33" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E33" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
@@ -1249,11 +1267,14 @@
       <c r="B34" t="s">
         <v>25</v>
       </c>
+      <c r="C34" t="s">
+        <v>127</v>
+      </c>
       <c r="D34" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E34" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
@@ -1264,10 +1285,10 @@
         <v>26</v>
       </c>
       <c r="D35" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E35" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
@@ -1278,10 +1299,10 @@
         <v>27</v>
       </c>
       <c r="D36" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E36" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
@@ -1292,21 +1313,21 @@
         <v>28</v>
       </c>
       <c r="E37" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B38" t="s">
         <v>29</v>
       </c>
       <c r="D38" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E38" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -1317,27 +1338,27 @@
         <v>36</v>
       </c>
       <c r="D39" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E39" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B40" t="s">
         <v>32</v>
       </c>
       <c r="D40" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E40" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F40" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
@@ -1345,13 +1366,13 @@
         <v>70</v>
       </c>
       <c r="B41" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D41" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E41" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>